<commit_message>
[scrum master] sprint 6
</commit_message>
<xml_diff>
--- a/SE202526/Management/WorkBreakdownStructure.xlsx
+++ b/SE202526/Management/WorkBreakdownStructure.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Uni\ES\SE2526_66565_67196_67215_68509_68663_70116\SE202526\Management\Sprint1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raksh\Documents\Git\projeto\SE2526_66565_67196_67215_68509_68663_70116\SE202526\Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9188C1-1F17-4925-B935-3C55EDCC2DC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32537F2A-88F6-4350-AAC4-59F14B4E4449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{069D515D-B00E-43A8-B28D-C4CC38ED1BD3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{069D515D-B00E-43A8-B28D-C4CC38ED1BD3}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="1" r:id="rId1"/>
     <sheet name="Week 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Week6" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>All members must explore the source code</t>
   </si>
@@ -61,6 +62,21 @@
   </si>
   <si>
     <t>Write the 3 user stories according to the given template</t>
+  </si>
+  <si>
+    <t>Sprint 6</t>
+  </si>
+  <si>
+    <t>Conclusion and review of documentation of US1, US2</t>
+  </si>
+  <si>
+    <t>Conclusion of the implementation of US3</t>
+  </si>
+  <si>
+    <t>Code improvement US1, US2</t>
+  </si>
+  <si>
+    <t>Documentation US3</t>
   </si>
 </sst>
 </file>
@@ -76,7 +92,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -86,6 +102,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -102,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -110,6 +132,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,28 +468,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D024881-D910-493D-9304-11EC0A5ED581}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="55.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="55.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -479,29 +502,67 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C11F634-1581-4049-B8FA-8868616056F4}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="54.85546875" customWidth="1"/>
+    <col min="1" max="1" width="54.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C08106C8-0437-46B0-B1D9-EA5161B1764F}">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="42.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added sprint 4 to WorkBreakdownStructure.xlsx
</commit_message>
<xml_diff>
--- a/SE202526/Management/WorkBreakdownStructure.xlsx
+++ b/SE202526/Management/WorkBreakdownStructure.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raksh\Documents\Git\projeto\SE2526_66565_67196_67215_68509_68663_70116\SE202526\Management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SE2526_66565_67196_67215_68509_68663_70116\SE202526\Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32537F2A-88F6-4350-AAC4-59F14B4E4449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{427881F0-5B39-4A83-BFAF-A99605AFA6F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{069D515D-B00E-43A8-B28D-C4CC38ED1BD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{069D515D-B00E-43A8-B28D-C4CC38ED1BD3}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="1" r:id="rId1"/>
     <sheet name="Week 2" sheetId="2" r:id="rId2"/>
-    <sheet name="Week6" sheetId="3" r:id="rId3"/>
+    <sheet name="Week 4" sheetId="4" r:id="rId3"/>
+    <sheet name="Week6" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>All members must explore the source code</t>
   </si>
@@ -64,9 +65,6 @@
     <t>Write the 3 user stories according to the given template</t>
   </si>
   <si>
-    <t>Sprint 6</t>
-  </si>
-  <si>
     <t>Conclusion and review of documentation of US1, US2</t>
   </si>
   <si>
@@ -77,6 +75,21 @@
   </si>
   <si>
     <t>Documentation US3</t>
+  </si>
+  <si>
+    <t>Week6</t>
+  </si>
+  <si>
+    <t>Week4</t>
+  </si>
+  <si>
+    <t>Each team should investigate the code relevant for their user story</t>
+  </si>
+  <si>
+    <t>Draft possible solutions for the problems found</t>
+  </si>
+  <si>
+    <t>Start implementing the user stories</t>
   </si>
 </sst>
 </file>
@@ -92,7 +105,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -102,12 +115,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -124,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -132,7 +139,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -151,7 +157,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -468,28 +474,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D024881-D910-493D-9304-11EC0A5ED581}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="55.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="55.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -502,27 +508,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C11F634-1581-4049-B8FA-8868616056F4}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="54.88671875" customWidth="1"/>
+    <col min="1" max="1" width="54.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -533,39 +539,84 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C08106C8-0437-46B0-B1D9-EA5161B1764F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C48BCB4-B6F5-462D-8E5B-43D35E4837AC}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.77734375" customWidth="1"/>
+    <col min="1" max="1" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C08106C8-0437-46B0-B1D9-EA5161B1764F}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="52.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added project demo video.
</commit_message>
<xml_diff>
--- a/SE202526/Management/WorkBreakdownStructure.xlsx
+++ b/SE202526/Management/WorkBreakdownStructure.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SE2526_66565_67196_67215_68509_68663_70116\SE202526\Management\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55D149A-9485-4097-8640-FC7FB468361C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Week 1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Week 2" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Week 3" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Week 4" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Week6" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Week 7" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Week 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Week 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Week 3" sheetId="3" r:id="rId3"/>
+    <sheet name="Week 4" sheetId="4" r:id="rId4"/>
+    <sheet name="Week6" sheetId="5" r:id="rId5"/>
+    <sheet name="Week 7" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,106 +30,94 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
-  <si>
-    <t xml:space="preserve">Week 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each member should play the game and think of a user story</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The group should pick the 3 best proposed user stories</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write the 3 user stories according to the given template</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All members must explore the source code</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Each member should play the game and think of a user story</t>
+  </si>
+  <si>
+    <t>The group should pick the 3 best proposed user stories</t>
+  </si>
+  <si>
+    <t>Write the 3 user stories according to the given template</t>
+  </si>
+  <si>
+    <t>All members must explore the source code</t>
   </si>
   <si>
     <t xml:space="preserve">Each one should find code smells in the code base  </t>
   </si>
   <si>
-    <t xml:space="preserve">The team report use cases and build a diagram around them</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All members must recognize 3 code smells and 3 design patterns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each member should create 5 use cases</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each member should create 1 use case diagram</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each team should investigate the code relevant for their user story</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Draft possible solutions for the problems found</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Start implementing the user stories</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conclusion and review of documentation of US1, US2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conclusion of the implementation of US3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code improvement US1, US2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentation US3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentation of US1, US2 and US3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review of the documentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Checks</t>
+    <t>The team report use cases and build a diagram around them</t>
+  </si>
+  <si>
+    <t>All members must recognize 3 code smells and 3 design patterns</t>
+  </si>
+  <si>
+    <t>Each member should create 5 use cases</t>
+  </si>
+  <si>
+    <t>Each member should create 1 use case diagram</t>
+  </si>
+  <si>
+    <t>Each team should investigate the code relevant for their user story</t>
+  </si>
+  <si>
+    <t>Draft possible solutions for the problems found</t>
+  </si>
+  <si>
+    <t>Start implementing the user stories</t>
+  </si>
+  <si>
+    <t>Conclusion and review of documentation of US1, US2</t>
+  </si>
+  <si>
+    <t>Conclusion of the implementation of US3</t>
+  </si>
+  <si>
+    <t>Code improvement US1, US2</t>
+  </si>
+  <si>
+    <t>Documentation US3</t>
+  </si>
+  <si>
+    <t>Documentation of US1, US2 and US3</t>
+  </si>
+  <si>
+    <t>Review of the documentation</t>
+  </si>
+  <si>
+    <t>Last Checks</t>
+  </si>
+  <si>
+    <t>Week 2</t>
+  </si>
+  <si>
+    <t>Week 3</t>
+  </si>
+  <si>
+    <t>Week 4</t>
+  </si>
+  <si>
+    <t>Week 6</t>
+  </si>
+  <si>
+    <t>Week 7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="3">
@@ -136,13 +129,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.7999"/>
+        <fgColor theme="7" tint="0.79989013336588644"/>
         <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -150,53 +143,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -255,60 +218,76 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0e2841"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e8e8e8"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="e97132"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196b24"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0f9ed5"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="a02b93"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4ea72e"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607d"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -340,7 +319,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -364,7 +343,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -424,290 +403,244 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="55.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="55.43"/>
+    <col min="1" max="1" width="55.140625" customWidth="1"/>
+    <col min="2" max="2" width="55.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="54.86"/>
+    <col min="1" max="1" width="54.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="61.28"/>
+    <col min="1" max="1" width="61.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
+    <col min="1" max="1" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52.72"/>
+    <col min="1" max="1" width="52.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52.72"/>
+    <col min="1" max="1" width="52.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added reviews to US2
</commit_message>
<xml_diff>
--- a/SE202526/Management/WorkBreakdownStructure.xlsx
+++ b/SE202526/Management/WorkBreakdownStructure.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SE2526_66565_67196_67215_68509_68663_70116\SE202526\Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55D149A-9485-4097-8640-FC7FB468361C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{743FA029-2274-45DC-BF80-F416BE0A09F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="1" r:id="rId1"/>
     <sheet name="Week 2" sheetId="2" r:id="rId2"/>
     <sheet name="Week 3" sheetId="3" r:id="rId3"/>
     <sheet name="Week 4" sheetId="4" r:id="rId4"/>
-    <sheet name="Week6" sheetId="5" r:id="rId5"/>
-    <sheet name="Week 7" sheetId="6" r:id="rId6"/>
+    <sheet name="Week 5" sheetId="7" r:id="rId5"/>
+    <sheet name="Week6" sheetId="5" r:id="rId6"/>
+    <sheet name="Week 7" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Week 1</t>
   </si>
@@ -105,6 +106,18 @@
   </si>
   <si>
     <t>Week 7</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>Implement User Story 1</t>
+  </si>
+  <si>
+    <t>Implement User Story 2</t>
+  </si>
+  <si>
+    <t>Discuss and begin to implement User Story 3</t>
   </si>
 </sst>
 </file>
@@ -554,6 +567,54 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{066CD53B-AC6B-416E-A7E7-182891094D2D}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="61.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -600,7 +661,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>